<commit_message>
- changed header text in Excel template - set value for NaN/Infinite
</commit_message>
<xml_diff>
--- a/api/templates/device_utilization_per_day/en.xlsx
+++ b/api/templates/device_utilization_per_day/en.xlsx
@@ -40,9 +40,6 @@
     <t>&lt;name&gt;</t>
   </si>
   <si>
-    <t>Device Capacity</t>
-  </si>
-  <si>
     <t>Total Results in period</t>
   </si>
   <si>
@@ -52,9 +49,6 @@
     <t>&lt;deviceCapacity&gt;</t>
   </si>
   <si>
-    <t>Utilization Rate</t>
-  </si>
-  <si>
     <t>&lt;utilizationRate&gt;</t>
   </si>
   <si>
@@ -62,6 +56,12 @@
   </si>
   <si>
     <t>Device Utilization per Day, number of tests</t>
+  </si>
+  <si>
+    <t>Daily Device Capacity</t>
+  </si>
+  <si>
+    <t>Utilization Rate (excluding weekends)</t>
   </si>
 </sst>
 </file>
@@ -616,13 +616,13 @@
   <cols>
     <col min="1" max="1" width="31.796875" customWidth="1"/>
     <col min="2" max="2" width="12.796875" customWidth="1"/>
-    <col min="3" max="3" width="10.59765625" customWidth="1"/>
-    <col min="4" max="4" width="10.3984375" style="1" customWidth="1"/>
+    <col min="3" max="3" width="12.69921875" customWidth="1"/>
+    <col min="4" max="4" width="21.3984375" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="21" x14ac:dyDescent="0.4">
       <c r="A1" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
@@ -653,13 +653,13 @@
         <v>3</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
@@ -667,13 +667,13 @@
         <v>5</v>
       </c>
       <c r="B8" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C8" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="D8" s="6" t="s">
         <v>9</v>
-      </c>
-      <c r="D8" s="6" t="s">
-        <v>11</v>
       </c>
     </row>
   </sheetData>
@@ -688,15 +688,14 @@
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="31.796875" style="1" customWidth="1"/>
-    <col min="2" max="2" width="12.796875" style="1" customWidth="1"/>
-    <col min="3" max="3" width="10.59765625" style="1" customWidth="1"/>
-    <col min="4" max="4" width="10.3984375" style="1" customWidth="1"/>
+    <col min="2" max="3" width="12.796875" style="1" customWidth="1"/>
+    <col min="4" max="4" width="21.296875" style="1" customWidth="1"/>
     <col min="5" max="16384" width="11" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="21" x14ac:dyDescent="0.4">
       <c r="A1" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
@@ -724,13 +723,13 @@
         <v>3</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
@@ -738,13 +737,13 @@
         <v>5</v>
       </c>
       <c r="B8" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C8" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="D8" s="6" t="s">
         <v>9</v>
-      </c>
-      <c r="D8" s="6" t="s">
-        <v>11</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
- add sub-headers in dynamic columns - process dynamic columns with spaned columns
</commit_message>
<xml_diff>
--- a/api/templates/device_utilization_per_day/en.xlsx
+++ b/api/templates/device_utilization_per_day/en.xlsx
@@ -126,7 +126,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -149,6 +149,35 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
@@ -195,7 +224,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -208,6 +237,15 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="43">
     <cellStyle name="Followed Hyperlink" xfId="2" builtinId="9" hidden="1"/>
@@ -617,7 +655,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="31.796875" customWidth="1"/>
@@ -653,36 +691,51 @@
       <c r="A6" s="1" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="7" spans="1:4" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="3" t="s">
+      <c r="B6">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="19.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="C7" s="7" t="s">
+      <c r="C7" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="D7" s="7" t="s">
+      <c r="D7" s="11" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A8" s="4" t="s">
+      <c r="A8" s="9"/>
+      <c r="B8" s="9"/>
+      <c r="C8" s="9"/>
+      <c r="D8" s="12"/>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A9" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B9" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="C9" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="D8" s="6" t="s">
+      <c r="D9" s="6" t="s">
         <v>9</v>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="A7:A8"/>
+    <mergeCell ref="B7:B8"/>
+    <mergeCell ref="C7:C8"/>
+    <mergeCell ref="D7:D8"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
leave only 1st sheet in Excel
</commit_message>
<xml_diff>
--- a/api/templates/device_utilization_per_day/en.xlsx
+++ b/api/templates/device_utilization_per_day/en.xlsx
@@ -12,15 +12,14 @@
     <workbookView xWindow="35568" yWindow="1332" windowWidth="22992" windowHeight="16080" tabRatio="815"/>
   </bookViews>
   <sheets>
-    <sheet name="Utilization Raw Data" sheetId="1" r:id="rId1"/>
-    <sheet name="Utilization Percentage" sheetId="2" r:id="rId2"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="162913" fullPrecision="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
     <t>&lt;Table&gt;</t>
   </si>
@@ -28,15 +27,9 @@
     <t>Dates: &lt;Dates&gt;</t>
   </si>
   <si>
-    <t>States: &lt;States&gt;</t>
-  </si>
-  <si>
     <t>Device</t>
   </si>
   <si>
-    <t>LGA: &lt;Lgas&gt;</t>
-  </si>
-  <si>
     <t>&lt;name&gt;</t>
   </si>
   <si>
@@ -52,12 +45,6 @@
     <t>&lt;utilizationRate&gt;</t>
   </si>
   <si>
-    <t>Device Utilization per Day, percentage</t>
-  </si>
-  <si>
-    <t>Device Utilization per Day, number of tests</t>
-  </si>
-  <si>
     <t>Daily Device Capacity</t>
   </si>
   <si>
@@ -68,6 +55,9 @@
   </si>
   <si>
     <t>&lt;LgasLabel&gt;: &lt;Lgas&gt;</t>
+  </si>
+  <si>
+    <t>Device Utilization per Day, number of tests and percentage</t>
   </si>
 </sst>
 </file>
@@ -126,27 +116,12 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="4">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color auto="1"/>
-      </left>
-      <right style="medium">
-        <color auto="1"/>
-      </right>
-      <top style="medium">
-        <color auto="1"/>
-      </top>
-      <bottom style="medium">
-        <color auto="1"/>
-      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -224,28 +199,21 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="43">
     <cellStyle name="Followed Hyperlink" xfId="2" builtinId="9" hidden="1"/>
@@ -666,7 +634,7 @@
   <sheetData>
     <row r="1" spans="1:4" ht="21" x14ac:dyDescent="0.4">
       <c r="A1" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
@@ -676,12 +644,12 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
@@ -696,37 +664,37 @@
       </c>
     </row>
     <row r="7" spans="1:4" ht="19.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="8" t="s">
+      <c r="A7" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D7" s="8" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A8" s="6"/>
+      <c r="B8" s="6"/>
+      <c r="C8" s="6"/>
+      <c r="D8" s="9"/>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A9" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B7" s="10" t="s">
+      <c r="B9" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C9" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C7" s="10" t="s">
-        <v>12</v>
-      </c>
-      <c r="D7" s="11" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A8" s="9"/>
-      <c r="B8" s="9"/>
-      <c r="C8" s="9"/>
-      <c r="D8" s="12"/>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A9" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="B9" s="4" t="s">
+      <c r="D9" s="4" t="s">
         <v>7</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D9" s="6" t="s">
-        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -739,74 +707,4 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" orientation="portrait" r:id="rId1"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D8"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="31.796875" style="1" customWidth="1"/>
-    <col min="2" max="3" width="12.796875" style="1" customWidth="1"/>
-    <col min="4" max="4" width="21.296875" style="1" customWidth="1"/>
-    <col min="5" max="16384" width="11" style="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:4" ht="21" x14ac:dyDescent="0.4">
-      <c r="A1" s="2" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A3" s="1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A4" s="1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B7" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="C7" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="D7" s="7" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A8" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D8" s="6" t="s">
-        <v>9</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup fitToHeight="0" orientation="portrait" r:id="rId1"/>
-</worksheet>
 </file>
</xml_diff>